<commit_message>
Add fully-passing Excel reports from GitHub Actions
Both suites now pass 15/15 on GitHub's own infrastructure (run
33847882829 for Appium against a real emulator, 33847882843 for
Selenium) — these are the real generated reports from those runs,
downloaded and committed here so they're visible and downloadable
directly from the repo, not just as time-limited CI artifacts.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/e2e-web/reports/selenium-report.xlsx
+++ b/e2e-web/reports/selenium-report.xlsx
@@ -128,19 +128,19 @@
     <t>Run Started (UTC)</t>
   </si>
   <si>
-    <t>2026-09-04T05:36:14.456Z</t>
+    <t>2026-09-04T07:16:54.367Z</t>
   </si>
   <si>
     <t>Run Ended (UTC)</t>
   </si>
   <si>
-    <t>2026-09-04T05:37:05.874Z</t>
+    <t>2026-09-04T07:17:25.027Z</t>
   </si>
   <si>
     <t>Report Generated (UTC)</t>
   </si>
   <si>
-    <t>2026-09-04T05:37:05.875Z</t>
+    <t>2026-09-04T07:17:25.028Z</t>
   </si>
 </sst>
 </file>
@@ -560,7 +560,7 @@
         <v>6</v>
       </c>
       <c r="D2">
-        <v>42</v>
+        <v>47</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -574,7 +574,7 @@
         <v>6</v>
       </c>
       <c r="D3">
-        <v>85</v>
+        <v>73</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -588,7 +588,7 @@
         <v>6</v>
       </c>
       <c r="D4">
-        <v>151</v>
+        <v>187</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -602,7 +602,7 @@
         <v>6</v>
       </c>
       <c r="D5">
-        <v>555</v>
+        <v>626</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -616,7 +616,7 @@
         <v>6</v>
       </c>
       <c r="D6">
-        <v>120</v>
+        <v>102</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -630,7 +630,7 @@
         <v>6</v>
       </c>
       <c r="D7">
-        <v>107</v>
+        <v>54</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -644,7 +644,7 @@
         <v>6</v>
       </c>
       <c r="D8">
-        <v>113</v>
+        <v>72</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -658,7 +658,7 @@
         <v>6</v>
       </c>
       <c r="D9">
-        <v>81</v>
+        <v>59</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -672,7 +672,7 @@
         <v>6</v>
       </c>
       <c r="D10">
-        <v>1215</v>
+        <v>1118</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -686,7 +686,7 @@
         <v>6</v>
       </c>
       <c r="D11">
-        <v>6379</v>
+        <v>6275</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -700,7 +700,7 @@
         <v>6</v>
       </c>
       <c r="D12">
-        <v>225</v>
+        <v>132</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -714,7 +714,7 @@
         <v>6</v>
       </c>
       <c r="D13">
-        <v>293</v>
+        <v>199</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -728,7 +728,7 @@
         <v>6</v>
       </c>
       <c r="D14">
-        <v>376</v>
+        <v>293</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -742,7 +742,7 @@
         <v>6</v>
       </c>
       <c r="D15">
-        <v>264</v>
+        <v>283</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -756,7 +756,7 @@
         <v>6</v>
       </c>
       <c r="D16">
-        <v>490</v>
+        <v>126</v>
       </c>
     </row>
   </sheetData>
@@ -820,7 +820,7 @@
         <v>34</v>
       </c>
       <c r="B6">
-        <v>10496</v>
+        <v>9646</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -828,7 +828,7 @@
         <v>35</v>
       </c>
       <c r="B7">
-        <v>51418</v>
+        <v>30660</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>